<commit_message>
added week 7 timesheets
</commit_message>
<xml_diff>
--- a/Documentation/Week 7/Booked Hours/Booked_Hours_Dylan.xlsx
+++ b/Documentation/Week 7/Booked Hours/Booked_Hours_Dylan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniwa-my.sharepoint.com/personal/24314441_student_uwa_edu_au/Documents/UWA/Year 3/Sem 2/CITS3200_Project/Documentation/Week 7/Booked Hours/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="248" documentId="8_{C839D0D7-89B3-4B1F-A7FA-FAF46048CC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D50DF943-6F3E-4682-B881-E1497D024A9F}"/>
+  <xr:revisionPtr revIDLastSave="275" documentId="8_{C839D0D7-89B3-4B1F-A7FA-FAF46048CC2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC1D6907-F7F4-4069-AF02-04C84EA055DF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="26">
   <si>
     <r>
       <t xml:space="preserve">CITS3200 Project Billed Hours Record for &lt;Dylan Hu&gt;
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t xml:space="preserve">Coding and debugging </t>
+  </si>
+  <si>
+    <t>Project testing and debugging</t>
   </si>
 </sst>
 </file>
@@ -820,7 +823,7 @@
     <col min="6" max="6" width="64.6328125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.36328125" style="1" customWidth="1"/>
     <col min="8" max="8" width="10.6328125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="0.36328125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="0.1796875" style="1" customWidth="1"/>
     <col min="10" max="16384" width="10.6328125" style="1"/>
   </cols>
   <sheetData>
@@ -964,7 +967,7 @@
         <v>1.5</v>
       </c>
       <c r="H6" s="1">
-        <f t="shared" ref="H6:H27" si="2">IF(AND(G6&lt;&gt;" ",G6&lt;&gt;"ERROR",H5&lt;&gt;" ", H5&lt;&gt;"ERROR"),G6+H5," ")</f>
+        <f t="shared" ref="H6:H28" si="2">IF(AND(G6&lt;&gt;" ",G6&lt;&gt;"ERROR",H5&lt;&gt;" ", H5&lt;&gt;"ERROR"),G6+H5," ")</f>
         <v>3.2499999999417923</v>
       </c>
       <c r="I6" s="1">
@@ -1645,15 +1648,67 @@
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="I28" s="1" t="e">
-        <f>((#REF!+#REF!)-(#REF!+#REF!))*24</f>
-        <v>#REF!</v>
+      <c r="A28" s="1">
+        <v>7</v>
+      </c>
+      <c r="B28" s="4">
+        <v>44816</v>
+      </c>
+      <c r="C28" s="5">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D28" s="4">
+        <v>44816</v>
+      </c>
+      <c r="E28" s="5">
+        <v>0.67708333333333337</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" s="6">
+        <f t="shared" si="0"/>
+        <v>0.25000000011641532</v>
+      </c>
+      <c r="H28" s="1">
+        <f t="shared" si="2"/>
+        <v>25.499999999825377</v>
+      </c>
+      <c r="I28" s="1">
+        <f>((D28+E28)-(B28+C28))*24</f>
+        <v>0.25000000011641532</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="I29" s="1" t="e">
-        <f>((#REF!+#REF!)-(#REF!+#REF!))*24</f>
-        <v>#REF!</v>
+      <c r="A29" s="1">
+        <v>8</v>
+      </c>
+      <c r="B29" s="4">
+        <v>44817</v>
+      </c>
+      <c r="C29" s="5">
+        <v>0.67708333333333337</v>
+      </c>
+      <c r="D29" s="4">
+        <v>44817</v>
+      </c>
+      <c r="E29" s="5">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G29" s="6">
+        <f t="shared" ref="G29" si="7">IF(I29&gt;0,I29,IF(I29=0, " ", "ERROR"))</f>
+        <v>0.75</v>
+      </c>
+      <c r="H29" s="1">
+        <f t="shared" ref="H29" si="8">IF(AND(G29&lt;&gt;" ",G29&lt;&gt;"ERROR",H28&lt;&gt;" ", H28&lt;&gt;"ERROR"),G29+H28," ")</f>
+        <v>26.249999999825377</v>
+      </c>
+      <c r="I29" s="1">
+        <f>((D29+E29)-(B29+C29))*24</f>
+        <v>0.75</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
@@ -1665,10 +1720,6 @@
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="H30" s="1" t="e">
-        <f>IF(AND(G30&lt;&gt;" ",G30&lt;&gt;"ERROR",#REF!&lt;&gt;" ",#REF!&lt;&gt; "ERROR"),G30+#REF!," ")</f>
-        <v>#REF!</v>
-      </c>
       <c r="I30" s="1">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -1728,12 +1779,12 @@
       <c r="D33" s="4"/>
       <c r="E33" s="5"/>
       <c r="G33" s="6" t="str">
-        <f t="shared" ref="G33:G64" si="7">IF(I33&gt;0,I33,IF(I33=0, " ", "ERROR"))</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H33" s="1" t="e">
+        <f t="shared" ref="G33:G64" si="9">IF(I33&gt;0,I33,IF(I33=0, " ", "ERROR"))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H33" s="1" t="str">
         <f>IF(AND(G33&lt;&gt;" ",G33&lt;&gt;"ERROR",H30&lt;&gt;" ", H30&lt;&gt;"ERROR"),G33+H30," ")</f>
-        <v>#REF!</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I33" s="1">
         <f t="shared" si="1"/>
@@ -1746,12 +1797,12 @@
       <c r="D34" s="4"/>
       <c r="E34" s="5"/>
       <c r="G34" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H34" s="1" t="e">
-        <f t="shared" ref="H34:H64" si="8">IF(AND(G34&lt;&gt;" ",G34&lt;&gt;"ERROR",H33&lt;&gt;" ", H33&lt;&gt;"ERROR"),G34+H33," ")</f>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H34" s="1" t="str">
+        <f t="shared" ref="H34:H64" si="10">IF(AND(G34&lt;&gt;" ",G34&lt;&gt;"ERROR",H33&lt;&gt;" ", H33&lt;&gt;"ERROR"),G34+H33," ")</f>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I34" s="1">
         <f t="shared" si="1"/>
@@ -1764,12 +1815,12 @@
       <c r="D35" s="4"/>
       <c r="E35" s="5"/>
       <c r="G35" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H35" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H35" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I35" s="1">
         <f t="shared" si="1"/>
@@ -1782,12 +1833,12 @@
       <c r="D36" s="4"/>
       <c r="E36" s="5"/>
       <c r="G36" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H36" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H36" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I36" s="1">
         <f t="shared" si="1"/>
@@ -1800,12 +1851,12 @@
       <c r="D37" s="4"/>
       <c r="E37" s="5"/>
       <c r="G37" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H37" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H37" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I37" s="1">
         <f t="shared" si="1"/>
@@ -1818,12 +1869,12 @@
       <c r="D38" s="4"/>
       <c r="E38" s="5"/>
       <c r="G38" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H38" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H38" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I38" s="1">
         <f t="shared" si="1"/>
@@ -1836,12 +1887,12 @@
       <c r="D39" s="4"/>
       <c r="E39" s="5"/>
       <c r="G39" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H39" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H39" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I39" s="1">
         <f t="shared" si="1"/>
@@ -1854,12 +1905,12 @@
       <c r="D40" s="4"/>
       <c r="E40" s="5"/>
       <c r="G40" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H40" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H40" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I40" s="1">
         <f t="shared" si="1"/>
@@ -1872,12 +1923,12 @@
       <c r="D41" s="4"/>
       <c r="E41" s="5"/>
       <c r="G41" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H41" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H41" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I41" s="1">
         <f t="shared" si="1"/>
@@ -1890,12 +1941,12 @@
       <c r="D42" s="4"/>
       <c r="E42" s="5"/>
       <c r="G42" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H42" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H42" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I42" s="1">
         <f t="shared" si="1"/>
@@ -1908,12 +1959,12 @@
       <c r="D43" s="4"/>
       <c r="E43" s="5"/>
       <c r="G43" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H43" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H43" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I43" s="1">
         <f t="shared" si="1"/>
@@ -1926,12 +1977,12 @@
       <c r="D44" s="4"/>
       <c r="E44" s="5"/>
       <c r="G44" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H44" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H44" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I44" s="1">
         <f t="shared" si="1"/>
@@ -1944,12 +1995,12 @@
       <c r="D45" s="4"/>
       <c r="E45" s="5"/>
       <c r="G45" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H45" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H45" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I45" s="1">
         <f t="shared" si="1"/>
@@ -1962,12 +2013,12 @@
       <c r="D46" s="4"/>
       <c r="E46" s="5"/>
       <c r="G46" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H46" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H46" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I46" s="1">
         <f t="shared" si="1"/>
@@ -1980,12 +2031,12 @@
       <c r="D47" s="4"/>
       <c r="E47" s="5"/>
       <c r="G47" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H47" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H47" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I47" s="1">
         <f t="shared" si="1"/>
@@ -1998,12 +2049,12 @@
       <c r="D48" s="4"/>
       <c r="E48" s="5"/>
       <c r="G48" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H48" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H48" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I48" s="1">
         <f t="shared" si="1"/>
@@ -2016,12 +2067,12 @@
       <c r="D49" s="4"/>
       <c r="E49" s="5"/>
       <c r="G49" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H49" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H49" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I49" s="1">
         <f t="shared" si="1"/>
@@ -2034,12 +2085,12 @@
       <c r="D50" s="4"/>
       <c r="E50" s="5"/>
       <c r="G50" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H50" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H50" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I50" s="1">
         <f t="shared" si="1"/>
@@ -2052,12 +2103,12 @@
       <c r="D51" s="4"/>
       <c r="E51" s="5"/>
       <c r="G51" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H51" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H51" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I51" s="1">
         <f t="shared" si="1"/>
@@ -2070,12 +2121,12 @@
       <c r="D52" s="4"/>
       <c r="E52" s="5"/>
       <c r="G52" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H52" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H52" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I52" s="1">
         <f t="shared" si="1"/>
@@ -2088,12 +2139,12 @@
       <c r="D53" s="4"/>
       <c r="E53" s="5"/>
       <c r="G53" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H53" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H53" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I53" s="1">
         <f t="shared" si="1"/>
@@ -2106,12 +2157,12 @@
       <c r="D54" s="4"/>
       <c r="E54" s="5"/>
       <c r="G54" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H54" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H54" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I54" s="1">
         <f t="shared" si="1"/>
@@ -2124,12 +2175,12 @@
       <c r="D55" s="4"/>
       <c r="E55" s="5"/>
       <c r="G55" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H55" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H55" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I55" s="1">
         <f t="shared" si="1"/>
@@ -2142,12 +2193,12 @@
       <c r="D56" s="4"/>
       <c r="E56" s="5"/>
       <c r="G56" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H56" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H56" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I56" s="1">
         <f t="shared" si="1"/>
@@ -2160,12 +2211,12 @@
       <c r="D57" s="4"/>
       <c r="E57" s="5"/>
       <c r="G57" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H57" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H57" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I57" s="1">
         <f t="shared" si="1"/>
@@ -2178,12 +2229,12 @@
       <c r="D58" s="4"/>
       <c r="E58" s="5"/>
       <c r="G58" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H58" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H58" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I58" s="1">
         <f t="shared" si="1"/>
@@ -2196,12 +2247,12 @@
       <c r="D59" s="4"/>
       <c r="E59" s="5"/>
       <c r="G59" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H59" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H59" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I59" s="1">
         <f t="shared" si="1"/>
@@ -2211,12 +2262,12 @@
     <row r="60" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B60" s="4"/>
       <c r="G60" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H60" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H60" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I60" s="1">
         <f t="shared" si="1"/>
@@ -2226,12 +2277,12 @@
     <row r="61" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B61" s="4"/>
       <c r="G61" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H61" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H61" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I61" s="1">
         <f t="shared" si="1"/>
@@ -2241,12 +2292,12 @@
     <row r="62" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B62" s="4"/>
       <c r="G62" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H62" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H62" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I62" s="1">
         <f t="shared" si="1"/>
@@ -2256,12 +2307,12 @@
     <row r="63" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B63" s="4"/>
       <c r="G63" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H63" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H63" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I63" s="1">
         <f t="shared" si="1"/>
@@ -2271,12 +2322,12 @@
     <row r="64" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B64" s="4"/>
       <c r="G64" s="6" t="str">
-        <f t="shared" si="7"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H64" s="1" t="e">
-        <f t="shared" si="8"/>
-        <v>#REF!</v>
+        <f t="shared" si="9"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H64" s="1" t="str">
+        <f t="shared" si="10"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I64" s="1">
         <f t="shared" si="1"/>
@@ -2333,12 +2384,12 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G67" s="6" t="str">
-        <f t="shared" ref="G67:G98" si="9">IF(I67&gt;0,I67,IF(I67=0, " ", "ERROR"))</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H67" s="1" t="e">
+        <f t="shared" ref="G67:G98" si="11">IF(I67&gt;0,I67,IF(I67=0, " ", "ERROR"))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H67" s="1" t="str">
         <f>IF(AND(G67&lt;&gt;" ",G67&lt;&gt;"ERROR",H64&lt;&gt;" ", H64&lt;&gt;"ERROR"),G67+H64," ")</f>
-        <v>#REF!</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I67" s="1">
         <f t="shared" si="1"/>
@@ -2347,12 +2398,12 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G68" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H68" s="1" t="e">
-        <f t="shared" ref="H68:H98" si="10">IF(AND(G68&lt;&gt;" ",G68&lt;&gt;"ERROR",H67&lt;&gt;" ", H67&lt;&gt;"ERROR"),G68+H67," ")</f>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H68" s="1" t="str">
+        <f t="shared" ref="H68:H98" si="12">IF(AND(G68&lt;&gt;" ",G68&lt;&gt;"ERROR",H67&lt;&gt;" ", H67&lt;&gt;"ERROR"),G68+H67," ")</f>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I68" s="1">
         <f t="shared" si="1"/>
@@ -2361,421 +2412,421 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G69" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H69" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H69" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I69" s="1">
-        <f t="shared" ref="I69:I132" si="11">((D69+E69)-(B69+C69))*24</f>
+        <f t="shared" ref="I69:I132" si="13">((D69+E69)-(B69+C69))*24</f>
         <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G70" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H70" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H70" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I70" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G71" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H71" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H71" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I71" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G72" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H72" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H72" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I72" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G73" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H73" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H73" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I73" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G74" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H74" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H74" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I74" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G75" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H75" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H75" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I75" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G76" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H76" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H76" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I76" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G77" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H77" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H77" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I77" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G78" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H78" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H78" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I78" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G79" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H79" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H79" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I79" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G80" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H80" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H80" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I80" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="81" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G81" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H81" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H81" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I81" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="82" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G82" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H82" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H82" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I82" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="83" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G83" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H83" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H83" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I83" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="84" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G84" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H84" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H84" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I84" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="85" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G85" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H85" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H85" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I85" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="86" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G86" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H86" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H86" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I86" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="87" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G87" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H87" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H87" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I87" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="88" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G88" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H88" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H88" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I88" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="89" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G89" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H89" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H89" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I89" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="90" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G90" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H90" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H90" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I90" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="91" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G91" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H91" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H91" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I91" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="92" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G92" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H92" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H92" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I92" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="93" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G93" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H93" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H93" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I93" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="94" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G94" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H94" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H94" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I94" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="95" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G95" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H95" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H95" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I95" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="96" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G96" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H96" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H96" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I96" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G97" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H97" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H97" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I97" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G98" s="6" t="str">
-        <f t="shared" si="9"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H98" s="1" t="e">
-        <f t="shared" si="10"/>
-        <v>#REF!</v>
+        <f t="shared" si="11"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H98" s="1" t="str">
+        <f t="shared" si="12"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I98" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
@@ -2801,7 +2852,7 @@
         <v>6</v>
       </c>
       <c r="I99" s="1" t="e">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>#VALUE!</v>
       </c>
     </row>
@@ -2823,455 +2874,455 @@
       <c r="G100" s="8"/>
       <c r="H100" s="8"/>
       <c r="I100" s="1" t="e">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G101" s="6" t="str">
-        <f t="shared" ref="G101:G132" si="12">IF(I101&gt;0,I101,IF(I101=0, " ", "ERROR"))</f>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H101" s="1" t="e">
+        <f t="shared" ref="G101:G132" si="14">IF(I101&gt;0,I101,IF(I101=0, " ", "ERROR"))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H101" s="1" t="str">
         <f>IF(AND(G101&lt;&gt;" ",G101&lt;&gt;"ERROR",H98&lt;&gt;" ", H98&lt;&gt;"ERROR"),G101+H98," ")</f>
-        <v>#REF!</v>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I101" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G102" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H102" s="1" t="e">
-        <f t="shared" ref="H102:H132" si="13">IF(AND(G102&lt;&gt;" ",G102&lt;&gt;"ERROR",H101&lt;&gt;" ", H101&lt;&gt;"ERROR"),G102+H101," ")</f>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H102" s="1" t="str">
+        <f t="shared" ref="H102:H132" si="15">IF(AND(G102&lt;&gt;" ",G102&lt;&gt;"ERROR",H101&lt;&gt;" ", H101&lt;&gt;"ERROR"),G102+H101," ")</f>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I102" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G103" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H103" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H103" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I103" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G104" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H104" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H104" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I104" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G105" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H105" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H105" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I105" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G106" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H106" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H106" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I106" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G107" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H107" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H107" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I107" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G108" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H108" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H108" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I108" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G109" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H109" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H109" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I109" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G110" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H110" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H110" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I110" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G111" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H111" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H111" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I111" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.2">
       <c r="G112" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H112" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H112" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I112" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="113" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G113" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H113" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H113" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I113" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="114" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G114" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H114" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H114" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I114" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="115" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G115" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H115" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H115" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I115" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="116" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G116" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H116" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H116" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I116" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="117" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G117" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H117" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H117" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I117" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="118" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G118" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H118" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H118" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I118" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="119" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G119" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H119" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H119" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I119" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="120" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G120" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H120" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H120" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I120" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="121" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G121" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H121" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H121" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I121" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="122" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G122" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H122" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H122" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I122" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="123" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G123" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H123" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H123" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I123" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="124" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G124" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H124" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H124" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I124" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="125" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G125" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H125" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H125" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I125" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="126" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G126" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H126" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H126" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I126" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="127" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G127" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H127" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H127" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I127" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="128" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G128" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H128" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H128" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I128" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="129" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G129" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H129" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H129" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I129" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="130" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G130" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H130" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H130" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I130" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="131" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G131" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H131" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H131" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I131" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
     <row r="132" spans="7:9" x14ac:dyDescent="0.2">
       <c r="G132" s="6" t="str">
-        <f t="shared" si="12"/>
-        <v xml:space="preserve"> </v>
-      </c>
-      <c r="H132" s="1" t="e">
-        <f t="shared" si="13"/>
-        <v>#REF!</v>
+        <f t="shared" si="14"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H132" s="1" t="str">
+        <f t="shared" si="15"/>
+        <v xml:space="preserve"> </v>
       </c>
       <c r="I132" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>